<commit_message>
Update inventory for jeddah - 1782494826558
</commit_message>
<xml_diff>
--- a/stores/jeddah.xlsx
+++ b/stores/jeddah.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>Sno</t>
   </si>
@@ -30,6 +30,33 @@
   </si>
   <si>
     <t>Location</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>8886467080074</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2-3-1</t>
+  </si>
+  <si>
+    <t>6924526310020</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>3-6-4</t>
   </si>
 </sst>
 </file>
@@ -93,7 +120,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.71875" customWidth="true"/>
@@ -124,6 +151,46 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s" s="1">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s" s="1">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s" s="1">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="F2" t="s" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="1">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s" s="1">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Update inventory for jeddah - 1785306978728
</commit_message>
<xml_diff>
--- a/stores/jeddah.xlsx
+++ b/stores/jeddah.xlsx
@@ -190,6 +190,38 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t>8700216684705</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t>3-2-1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>